<commit_message>
feat: reorganiza financeiro por processo faturavel
</commit_message>
<xml_diff>
--- a/docs/spec/2026-08-12-behavioral-spec.xlsx
+++ b/docs/spec/2026-08-12-behavioral-spec.xlsx
@@ -2215,7 +2215,7 @@
         <v>Taxas Locais</v>
       </c>
       <c r="C57" t="str">
-        <v>As an admin I want /taxas-locais to manage charge tables, items and customer overrides</v>
+        <v>As an admin I want /taxas-locais/tabelas to manage charge tables, items and customer overrides</v>
       </c>
       <c r="D57" t="str">
         <v>TaxasLocais.tsx requires UI capabilities charge_tables/charge_overrides (useAuth); CRUD via chargeTableService.ts and chargeRateService.ts over charge_tables/charge_table_items/customer_rate_overrides (all admin-only at RLS); mutations invalidate queryKeys.charges.* families; table validity gates ready_for_billing.</v>
@@ -2230,10 +2230,10 @@
         <v>-</v>
       </c>
       <c r="H57" t="str">
-        <v>Vitest: TaxasLocais.behavior.test.tsx; TaxasLocais.test.ts; chargeRateService.test.ts; taxasLocaisHelpers.test.ts</v>
+        <v>Vitest: TaxasLocaisTabelas.test.ts; chargeRateService.test.ts; taxasLocaisHelpers.test.ts</v>
       </c>
       <c r="I57" t="str">
-        <v>src/pages/TaxasLocais.tsx; src/services/charges/chargeTableService.ts; src/services/charges/chargeRateService.ts</v>
+        <v>src/pages/TaxasLocaisTabelas.tsx; src/services/charges/chargeTableService.ts; src/services/charges/chargeRateService.ts</v>
       </c>
       <c r="J57" t="str">
         <v>-</v>
@@ -2695,10 +2695,10 @@
         <v>Faturamento</v>
       </c>
       <c r="C72" t="str">
-        <v>As a finance user I want /faturamento to validate B/Ls and manage the invoice lifecycle</v>
+        <v>As a finance user I want /taxas-locais to validate B/Ls and manage the invoice lifecycle</v>
       </c>
       <c r="D72" t="str">
-        <v>Faturamento.tsx (useBilling/useBillingLedger): validation/bottleneck view of B/Ls, individual and consolidated issuance, invoice list; InvoiceDetailModal registers payments, cancels, refunds and prints; all financial writes go through admin-guarded RPCs; caches for invoices/receivables/B/Ls/customers/alerts invalidated.</v>
+        <v>TaxasLocais.tsx (useBilling/useBillingLedger): validation/bottleneck view of B/Ls, individual and consolidated issuance, invoice list; InvoiceDetailModal registers payments, cancels, refunds and prints; all financial writes go through admin-guarded RPCs; caches for invoices/receivables/B/Ls/customers/alerts invalidated.</v>
       </c>
       <c r="E72" t="str">
         <v>Verified</v>
@@ -2710,10 +2710,10 @@
         <v>-</v>
       </c>
       <c r="H72" t="str">
-        <v>Vitest: Faturamento.behavior.test.tsx; Faturamento.test.ts; faturamentoInvoiceStatus.test.ts; faturamentoLedgerPayment.test.ts</v>
+        <v>Vitest: TaxasLocais.behavior.test.tsx; TaxasLocais.test.ts; faturamentoInvoiceStatus.test.ts; faturamentoLedgerPayment.test.ts</v>
       </c>
       <c r="I72" t="str">
-        <v>src/pages/Faturamento.tsx; src/services/billing.ts; src/services/billingLedger.ts</v>
+        <v>src/pages/TaxasLocais.tsx; src/services/billing.ts; src/services/billingLedger.ts</v>
       </c>
       <c r="J72" t="str">
         <v>-</v>
@@ -6076,7 +6076,7 @@
         <v>Source CSV</v>
       </c>
       <c r="B2" t="str">
-        <v>docs/spec/2026-08-12-behavioral-spec.csv</v>
+        <v>C:\Users\Lucca\Downloads\transhippingdesk\docs\spec\2026-08-12-behavioral-spec.csv</v>
       </c>
     </row>
     <row r="3">
@@ -6084,7 +6084,7 @@
         <v>Generated</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-08-12</v>
+        <v>2026-08-18</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
feat: implement bloco 5 de alertas do ADR
</commit_message>
<xml_diff>
--- a/docs/spec/2026-08-12-behavioral-spec.xlsx
+++ b/docs/spec/2026-08-12-behavioral-spec.xlsx
@@ -5802,7 +5802,7 @@
         <v>As a department I want to be alerted about a pending report and about a missed deadline, separately</v>
       </c>
       <c r="D169" t="str">
-        <v>detect_agency_report_pending() e detect_agency_report_deadline_missed() (migration 271) sao rotinas distintas: a pendencia e o vencimento do prazo geram alertas independentes, por departamento. O Prazo de Conclusao de tres dias uteis vem de uma funcao pura compartilhada entre tela, alerta e agregado.</v>
+        <v>detect_agency_report_pending() e detect_agency_report_deadline_missed() continuam produtores distintos, mas a migration 323 os reconcilia na fundação transversal: um agregado por ADR (voyage::port ou voyage::port::terminal) e dois itens independentes por departamento. O terminal usa terminal_atd; audit logs, sign-offs e o cron server-side de 15 minutos reprocessam a origem, com backfill sem notificações históricas. O prazo de três dias úteis continua vindo de uma função pura compartilhada entre tela, alerta e agregado.</v>
       </c>
       <c r="E169" t="str">
         <v>Verified</v>
@@ -5814,10 +5814,10 @@
         <v>-</v>
       </c>
       <c r="H169" t="str">
-        <v>Vitest: agencyReportSla.test.ts; agencyReportDeadline.test.ts; SQL-contract: agencyReportPendingAlertsMigration.test.ts; agencyReportDeadlineMissedMigration.test.ts</v>
+        <v>Vitest: agencyReportSla.test.ts; agencyReportDeadline.test.ts; SQL-contract: agencyReportPendingAlertsMigration.test.ts; agencyReportDeadlineMissedMigration.test.ts; agencyReportAlertsFoundationMigration.test.ts; runtime local PostgreSQL (323)</v>
       </c>
       <c r="I169" t="str">
-        <v>src/services/alerts.ts; src/services/agencyReportSla.ts; src/services/agencyReportDeadline.ts</v>
+        <v>src/services/alerts.ts; src/services/agencyReportSla.ts; src/services/agencyReportDeadline.ts; supabase/migrations/323_agency_report_alerts_foundation.sql</v>
       </c>
       <c r="J169" t="str">
         <v>-</v>
@@ -6076,7 +6076,7 @@
         <v>Source CSV</v>
       </c>
       <c r="B2" t="str">
-        <v>C:\Users\Lucca\Downloads\transhippingdesk\docs\spec\2026-08-12-behavioral-spec.csv</v>
+        <v>docs/spec/2026-08-12-behavioral-spec.csv</v>
       </c>
     </row>
     <row r="3">
@@ -6084,7 +6084,7 @@
         <v>Generated</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-08-18</v>
+        <v>2026-08-20</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
feat: integracao transversal dos blocos 520 a 524 (#519)
</commit_message>
<xml_diff>
--- a/docs/spec/2026-08-12-behavioral-spec.xlsx
+++ b/docs/spec/2026-08-12-behavioral-spec.xlsx
@@ -5802,7 +5802,7 @@
         <v>As a department I want to be alerted about a pending report and about a missed deadline, separately</v>
       </c>
       <c r="D169" t="str">
-        <v>detect_agency_report_pending() e detect_agency_report_deadline_missed() (migration 271) sao rotinas distintas: a pendencia e o vencimento do prazo geram alertas independentes, por departamento. O Prazo de Conclusao de tres dias uteis vem de uma funcao pura compartilhada entre tela, alerta e agregado.</v>
+        <v>detect_agency_report_pending() e detect_agency_report_deadline_missed() continuam produtores distintos, mas a migration 323 os reconcilia na fundação transversal: um agregado por ADR (voyage::port ou voyage::port::terminal) e dois itens independentes por departamento. O terminal usa terminal_atd; audit logs, sign-offs e o cron server-side de 15 minutos reprocessam a origem, com backfill sem notificações históricas. O prazo de três dias úteis continua vindo de uma função pura compartilhada entre tela, alerta e agregado.</v>
       </c>
       <c r="E169" t="str">
         <v>Verified</v>
@@ -5814,10 +5814,10 @@
         <v>-</v>
       </c>
       <c r="H169" t="str">
-        <v>Vitest: agencyReportSla.test.ts; agencyReportDeadline.test.ts; SQL-contract: agencyReportPendingAlertsMigration.test.ts; agencyReportDeadlineMissedMigration.test.ts</v>
+        <v>Vitest: agencyReportSla.test.ts; agencyReportDeadline.test.ts; SQL-contract: agencyReportPendingAlertsMigration.test.ts; agencyReportDeadlineMissedMigration.test.ts; agencyReportAlertsFoundationMigration.test.ts; runtime local PostgreSQL (323)</v>
       </c>
       <c r="I169" t="str">
-        <v>src/services/alerts.ts; src/services/agencyReportSla.ts; src/services/agencyReportDeadline.ts</v>
+        <v>src/services/alerts.ts; src/services/agencyReportSla.ts; src/services/agencyReportDeadline.ts; supabase/migrations/323_agency_report_alerts_foundation.sql</v>
       </c>
       <c r="J169" t="str">
         <v>-</v>
@@ -6076,7 +6076,7 @@
         <v>Source CSV</v>
       </c>
       <c r="B2" t="str">
-        <v>C:\Users\Lucca\Downloads\transhippingdesk\docs\spec\2026-08-12-behavioral-spec.csv</v>
+        <v>docs/spec/2026-08-12-behavioral-spec.csv</v>
       </c>
     </row>
     <row r="3">
@@ -6084,7 +6084,7 @@
         <v>Generated</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-08-18</v>
+        <v>2026-08-20</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
fix: corrigir comunicacoes financeiras do bloco 3
</commit_message>
<xml_diff>
--- a/docs/spec/2026-08-12-behavioral-spec.xlsx
+++ b/docs/spec/2026-08-12-behavioral-spec.xlsx
@@ -4327,10 +4327,10 @@
         <v>Portal / Faturamento</v>
       </c>
       <c r="C123" t="str">
-        <v>As the platform I can email the customer when an invoice is issued (currently inactive)</v>
+        <v>As the platform I can communicate a financially ready local-charge summary to the customer after CE Mercante is linked</v>
       </c>
       <c r="D123" t="str">
-        <v>notify-invoice-issued: bearer must equal SUPABASE_SERVICE_ROLE_KEY (timing-safe); accepts absent Origin or Origin == SUPABASE_URL; service role re-reads invoices/customers/customer_contacts (no DB writes) and sends via Resend; missing recipient/key -&gt; skipped/sent:false; auth failure 401; Resend/parse failure 500. No functions.invoke caller exists in src and no webhook is configured in the repo — inactive by decision; customer notification is in-app via trg_notify_invoice_issued.</v>
+        <v>customer_local_charges_communication_readiness(p_voyage_id,p_customer_id) requires an active internal reader and returns stable readiness reasons for every active B/L; send-customer-communication validates contacts/preferences/suppressions, records idempotent attempts and honors the global simulation switch. The ce_mercante_taxas template contains CE/B-L/BRL rows, voyage total and Portal link, without due date, PIX or attachments.</v>
       </c>
       <c r="E123" t="str">
         <v>Verified (static)</v>
@@ -4342,13 +4342,13 @@
         <v>-</v>
       </c>
       <c r="H123" t="str">
-        <v>Static</v>
+        <v>Static + Vitest: customerCommunicationReadinessMigration.test.ts; customerFinanceCommunications.test.ts</v>
       </c>
       <c r="I123" t="str">
-        <v>supabase/functions/notify-invoice-issued/index.ts</v>
+        <v>supabase/migrations/376_customer_local_charges_communication_readiness.sql; supabase/functions/send-customer-communication/index.ts</v>
       </c>
       <c r="J123" t="str">
-        <v>Inactive by decision (no webhook, no RESEND_API_KEY); reactivation is future work.</v>
+        <v>Automatic dispatch runs after CE linkage when all active B/Ls are ready; manual resend increments the discriminator.</v>
       </c>
     </row>
     <row r="124">
@@ -6084,7 +6084,7 @@
         <v>Generated</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-08-20</v>
+        <v>2026-09-01</v>
       </c>
     </row>
     <row r="4">

</xml_diff>